<commit_message>
Add --counties filter to enrichment script for PB/Broward focus
Filters leads by mailing address city before scoring. Includes
city lookup tables for Palm Beach and Broward counties. Re-ran
test with --counties "palm beach,broward": 7,537 qualifying leads,
top 25 all local LLCs with 5-29 properties.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scrape/data/enriched/research_tracker.xlsx
+++ b/scrape/data/enriched/research_tracker.xlsx
@@ -557,36 +557,32 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>JWC BERMUDA CAY LLC</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ROBBINS, STEVEN R</t>
-        </is>
-      </c>
+          <t>WORTHGATE APARTMENTS LLC</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1693500</t>
+          <t>770000</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>120 WELLS AVE, NEWTON CENTRE, MA 02459</t>
+          <t>PO BOX 904, DANIA, FL 33004</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>6177919349</t>
+          <t>9547796053</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -615,36 +611,32 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>DREA GROUP 28 LLC</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>PEREL MANAGEMENT, LLC</t>
-        </is>
-      </c>
+          <t>LAKE SHORE DEVELOPMENT LLC</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>908500</t>
+          <t>1885000</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>13322 SW 128TH ST, MIAMI, FL 33186</t>
+          <t>11231 US HIGHWAY 1 # 354, NORTH PALM BEACH, FL 33408</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>305.238.0600</t>
+          <t>5613369272</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -673,32 +665,32 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>NIGHT LION LLC</t>
+          <t>VERMONT APARTMENTS LLC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1100000</t>
+          <t>5534635</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>71 ELDORADO ST, ATLANTIC BEACH, NY 11509</t>
+          <t>7495 ATLANTIC AVE STE 200 112, DELRAY BEACH, FL 33446</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>5614532882</t>
+          <t>7252287035</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -727,32 +719,32 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>WPB MF LLC</t>
+          <t>FLORIDA ANGELS INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>5270224</t>
+          <t>9051875</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>251 LITTLE FALLS DR, WILMINGTON, DE 19808</t>
+          <t>1300 WOOD ROW WAY, WELLINGTON, FL 33414</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>561 833 6200</t>
+          <t>91758756800</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -781,36 +773,32 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>JWC BERMUDA CAY LLC</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>ROBBINS, STEVEN R</t>
-        </is>
-      </c>
+          <t>ROBERTS LANE LLC</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1126500</t>
+          <t>9222257</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>6830 PORTO FINO CIR, FORT MYERS, FL 33912</t>
+          <t>PO BOX 904, DANIA, FL 33004</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>6177919349</t>
+          <t>9547796053</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -839,32 +827,32 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>212NKST LLC</t>
+          <t>BEDFORD HOLDINGS LLC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1305000</t>
+          <t>3995765</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>3222 BRONXWOOD AVE, BRONX, NY 10469</t>
+          <t>PO BOX 3031, PALM BEACH, FL 33480</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>954-895-0517</t>
+          <t>561-429-8477</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -897,28 +885,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>BENNETT INVESTMENTS LLC</t>
+          <t>HRISTOV HOLDINGS LLC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1454347</t>
+          <t>5534560</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>515 N FLAGLER DR STE 1500, WEST PALM BEACH, FL 33401</t>
+          <t>1030 BIMINI LN, RIVIERA BEACH, FL 33404</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>6784921969</t>
+          <t>3032200183</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -951,30 +939,30 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>PACIFICA WEST PALM LLC</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>ISRANI, DEEPAK</t>
-        </is>
-      </c>
+          <t>BENNETT INVESTMENTS LLC</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1204000</t>
+          <t>1454347</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1775 HANCOCK ST STE 209, SAN DIEGO, CA 92110</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>515 N FLAGLER DR STE 1500, WEST PALM BEACH, FL 33401</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>6784921969</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -1005,28 +993,28 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TELMOUNT LLC</t>
+          <t>PB APARTMENTS 3 LLC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1449468</t>
+          <t>5845187</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>7 SHELDRAKE LN, PALM BCH GDNS, FL 33418</t>
+          <t>PO BOX 904, DANIA, FL 33004</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>561-838-5554</t>
+          <t>9547796053</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -1113,28 +1101,28 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>PB APARTMENTS 3 LLC</t>
+          <t>EXAGON INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>5845187</t>
+          <t>2047240</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>PO BOX 904, DANIA, FL 33004</t>
+          <t>304 INDIAN TRCE STE 507, WESTON, FL 33326</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>9547796053</t>
+          <t>9543491176</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1167,30 +1155,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ZAKAI LLC</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>HAKKI, FAWAZ Z</t>
-        </is>
-      </c>
+          <t>PICK LLC</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2159525</t>
+          <t>3575345</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>8535 HARPER DR, WAYNESBORO, PA 17268</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>3703 HERTFORD CT, GREENACRES, FL 33463</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>7866634790</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr">
         <is>
@@ -1221,28 +1209,28 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ATLANTIC AVE PROPERTIES LLC</t>
+          <t>MOON 921 LLC</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1813142</t>
+          <t>2937169</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1102 N ATLANTIC DR, LAKE WORTH, FL 33462</t>
+          <t>1059 SW 25TH AVE, BOYNTON BEACH, FL 33426</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>9175006417</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1275,30 +1263,30 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>AAG PROPERTY MANAGEMENT LLC</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>GURINO, ANTHONY</t>
-        </is>
-      </c>
+          <t>RAM BOCA RATON LLC</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1524926</t>
+          <t>11153645</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>8217 153RD AVE STE 206, JAMAICA, NY 11414</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>4156 NW 21ST AVE, FORT LAUDERDALE, FL 33309</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>9543684077</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr">
         <is>
@@ -1329,28 +1317,28 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>WALTON BLVD LLC</t>
+          <t>PB APARTMENTS 1 LLC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1328447</t>
+          <t>4203549</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>513 US HIGHWAY 1 STE 111, N PALM BEACH, FL 33408</t>
+          <t>PO BOX 904, DANIA, FL 33004</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>561.309.7228</t>
+          <t>9547796053</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1383,28 +1371,28 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>A &amp; Y APARTMENTS LLC</t>
+          <t>MA MAISON PROPERTY LLC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2285000</t>
+          <t>1660735</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1998 NE 7TH ST APT 106, DEERFIELD BEACH, FL 33441</t>
+          <t>PO BOX 880567, BOCA RATON, FL 33488</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>8589222282</t>
+          <t>2624971943</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1437,28 +1425,28 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>WORTHGATE APARTMENTS LLC</t>
+          <t>MERCER PARK HOMES LLC</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>770000</t>
+          <t>5470742</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>PO BOX 904, DANIA, FL 33004</t>
+          <t>251 OLEANDER AVE APT 3, PALM BEACH, FL 33480</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>9547796053</t>
+          <t>5708400201</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1491,28 +1479,28 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>GOLDEN GOOSE PROPERTIES INC</t>
+          <t>VENUS FLORIDA PROPERTIES LLC</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>9910457</t>
+          <t>1435227</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>3595 MIDDLEBURG DR, WELLINGTON, FL 33414</t>
+          <t>1200 N FEDERAL HWY STE 200, BOCA RATON, FL 33432</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>561.301.0388</t>
+          <t>7863800308</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1545,28 +1533,28 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>THL HOLDINGS LLC</t>
+          <t>SP APARTMENTS LLC</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>1095000</t>
+          <t>2700000</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>19521 SATURNIA LAKES DR, BOCA RATON, FL 33498</t>
+          <t>1913 A NW 40TH CT, POMPANO BEACH, FL 33064</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>6788777251</t>
+          <t>253-534-7200</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1599,14 +1587,10 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>RESICAP FLORIDA OWNER II LLC</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>RP Resicap Borrower II, LLC</t>
-        </is>
-      </c>
+          <t>A &amp; Y APARTMENTS LLC</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>22</t>
@@ -1614,15 +1598,19 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>9115440</t>
+          <t>2285000</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>3630 PEACHTREE RD NE STE 1500, ATLANTA, GA 30326</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>1998 NE 7TH ST APT 106, DEERFIELD BEACH, FL 33441</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>8589222282</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr">
         <is>
@@ -1653,28 +1641,28 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>SP APARTMENTS LLC</t>
+          <t>HOUSING PARTNERSHIP INC</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2700000</t>
+          <t>3866621</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1913 A NW 40TH CT, POMPANO BEACH, FL 33064</t>
+          <t>2001 W BLUE HERON BLVD, RIVIERA BEACH, FL 33404</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>253-534-7200</t>
+          <t>5618413500</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1707,28 +1695,28 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>BEG 3918 LLC</t>
+          <t>JL REALTY LLC</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>5082996</t>
+          <t>2958000</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>7984 ARBOR CREST WAY, PALM BEACH GARDENS, FL 33412</t>
+          <t>1000 N US HIGHWAY 1 APT 809, JUPITER, FL 33477</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>561-578-0203</t>
+          <t>3032200183</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1761,28 +1749,28 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CSA SEASCAPE LLC</t>
+          <t>WHITE ROSE HOMES LLC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>15179997</t>
+          <t>3949357</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>1541 SUNSET DR STE 300, MIAMI, FL 33143</t>
+          <t>PO BOX 1271, BOYNTON BEACH, FL 33425</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>561.844.5185</t>
+          <t>305.332.4332</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1815,26 +1803,30 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1111 N FEDERAL HWY REALTY LLC</t>
+          <t>GOLDEN GOOSE PROPERTIES INC</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>900000</t>
+          <t>9910457</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>3134 EMMONS AVE # 2, BROOKLYN, NY 11235</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>3595 MIDDLEBURG DR, WELLINGTON, FL 33414</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>561.301.0388</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr">
         <is>
@@ -1865,28 +1857,28 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>FIFTY FIVE HUNDRED FLAGLER LLC</t>
+          <t>MARCOS MANAGEMENT LLC</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>780000</t>
+          <t>1192500</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>251 SOUTHERN BLVD, WEST PALM BEACH, FL 33405</t>
+          <t>10870 CANYON BAY LN, BOYNTON BEACH, FL 33473</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>561.820.0090</t>
+          <t>561.843.5848</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>

</xml_diff>